<commit_message>
Core inflation, limit to years being shown, option to highlight variables added and data updated
</commit_message>
<xml_diff>
--- a/data/original/banco_republica/CPI/inflacion_15.xlsx
+++ b/data/original/banco_republica/CPI/inflacion_15.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="977">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1057" uniqueCount="979">
   <si>
     <t>Fecha</t>
   </si>
@@ -2900,10 +2900,16 @@
     <t>5,85</t>
   </si>
   <si>
+    <t>30/04/2026</t>
+  </si>
+  <si>
+    <t>5,87</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Descargado de sistema del Banco de la República martes, 5 de mayo de 2026 12:55:05 p. m.</t>
+    <t>Descargado de sistema del Banco de la República miércoles, 13 de mayo de 2026 4:17:35 p. m.</t>
   </si>
   <si>
     <t>Nombre de la serie</t>
@@ -3332,7 +3338,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B522"/>
+  <dimension ref="A1:B523"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -7491,19 +7497,27 @@
         <v>961</v>
       </c>
     </row>
-    <row r="520" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="520" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A520" t="s">
         <v>962</v>
       </c>
+      <c r="B520" t="s">
+        <v>963</v>
+      </c>
     </row>
     <row r="521" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A521" t="s">
-        <v>962</v>
+        <v>964</v>
       </c>
     </row>
     <row r="522" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A522" t="s">
-        <v>963</v>
+        <v>964</v>
+      </c>
+    </row>
+    <row r="523" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A523" t="s">
+        <v>965</v>
       </c>
     </row>
   </sheetData>
@@ -7526,48 +7540,48 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>964</v>
+        <v>966</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>965</v>
+        <v>967</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>966</v>
+        <v>968</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>967</v>
+        <v>969</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>968</v>
+        <v>970</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>969</v>
+        <v>971</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>970</v>
+        <v>972</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>971</v>
+        <v>973</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>972</v>
+        <v>974</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>973</v>
+        <v>975</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>974</v>
+        <v>976</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>975</v>
+        <v>977</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>976</v>
+        <v>978</v>
       </c>
     </row>
   </sheetData>

</xml_diff>